<commit_message>
Build q3011 content safety replay DAG migration
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R523e2839ec5d474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R1243d5d2a34a4903"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -306,7 +306,7 @@
         <x:v>辅助工具</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str">
-        <x:v>Python3.12、PyYAML6.0.2、UTF-8文本编辑器、CSV查看器、JSON查看器和YAML查看器</x:v>
+        <x:v>Python3.11、PyYAML6.0.2、UTF-8文本编辑器、CSV查看器、JSON查看器和YAML查看器</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">

</xml_diff>